<commit_message>
Add data analysis module and improve charts
Introduce analisis_datos.py (cargar_ingresos, top_impuestos_tributarios) and integrate it into app.py and motor_excel.py to compute top tributary revenue items dynamically. Refactor motor_excel: remove legacy test sheet, add/rename chart sheets (GRAFICOS), enhance BarChart configuration, styling, labels, axes and colors, and populate a second chart sheet using the top tributary items. Update requirements to include pandas. Binary artifacts updated: compiled .pyc files and outputs/CRUCE_FINAL.xlsx changed.
</commit_message>
<xml_diff>
--- a/outputs/CRUCE_FINAL.xlsx
+++ b/outputs/CRUCE_FINAL.xlsx
@@ -12,9 +12,8 @@
     <sheet name="CRUCE INFORMACION" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="REPORTE FILTRADO" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="INFORME RAPIDO" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="test" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="GRAFICOS" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="GRAF PRINCIPALES IMPUESTOS" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="GRAFICOS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="GRAF PRINCIPALES IMPUESTOS" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -343,131 +342,6 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>📊 Resumen de Esfuerzo Tributario Municipal</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="bar"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'REPORTE FILTRADO'!C1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="D9D9D9"/>
-            </a:solidFill>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'REPORTE FILTRADO'!$B$2:$B$8</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'REPORTE FILTRADO'!$C$2:$C$8</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'REPORTE FILTRADO'!D1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="00B050"/>
-            </a:solidFill>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'REPORTE FILTRADO'!$B$2:$B$8</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'REPORTE FILTRADO'!$D$2:$D$8</f>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <numFmt formatCode="$#,##0"/>
-          <showVal val="1"/>
-        </dLbls>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="maxMin"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="low"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="t"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-  <spPr>
-    <a:ln>
-      <a:noFill/>
-      <a:prstDash val="solid"/>
-    </a:ln>
-  </spPr>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
@@ -577,7 +451,6 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
@@ -585,7 +458,7 @@
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="t"/>
+      <legendPos val="l"/>
       <overlay val="0"/>
     </legend>
     <plotVisOnly val="1"/>
@@ -594,7 +467,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
@@ -704,7 +577,6 @@
         </scaling>
         <delete val="1"/>
         <axPos val="l"/>
-        <majorGridlines/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -756,7 +628,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10800000" cy="5760000"/>
+    <ext cx="13680000" cy="5760000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -775,33 +647,6 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="10080000" cy="5760000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -85518,20 +85363,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -85555,45 +85386,45 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Impuesto Predial Unificado</t>
+          <t>Impuesto Predial Unificado - Urbano</t>
         </is>
       </c>
       <c r="B2" s="10">
-        <f>INGRESOS!L9</f>
+        <f>INGRESOS!L10</f>
         <v/>
       </c>
       <c r="C2" s="10">
-        <f>INGRESOS!N9</f>
+        <f>INGRESOS!N10</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sobretasa a la gasolina</t>
+          <t>Impuesto de industria y comercio - sobre actividades comerciales</t>
         </is>
       </c>
       <c r="B3" s="10">
-        <f>INGRESOS!L13</f>
+        <f>INGRESOS!L15</f>
         <v/>
       </c>
       <c r="C3" s="10">
-        <f>INGRESOS!N13</f>
+        <f>INGRESOS!N15</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Impuesto de industria y comercio</t>
+          <t>Impuesto de alumbrado público</t>
         </is>
       </c>
       <c r="B4" s="10">
-        <f>INGRESOS!L14</f>
+        <f>INGRESOS!L19</f>
         <v/>
       </c>
       <c r="C4" s="10">
-        <f>INGRESOS!N14</f>
+        <f>INGRESOS!N19</f>
         <v/>
       </c>
     </row>

</xml_diff>